<commit_message>
literally just renaming stuff bro
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
@@ -910,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1.708002215362129e-09</v>
+        <v>1.730262261681266e-09</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>5.078618588555154e-08</v>
+        <v>5.109053708058755e-08</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>7.14457637652679e-07</v>
+        <v>7.151498059568239e-07</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>6.036736024256368e-06</v>
+        <v>6.026289630808105e-06</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>3.369823907655682e-05</v>
+        <v>3.361721063979729e-05</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0001331207389319273</v>
+        <v>0.0001328756464798305</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         <v>6</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0004017997448314381</v>
+        <v>0.0004012430301734141</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
         <v>7</v>
       </c>
       <c r="C34" t="n">
-        <v>0.001018529931036342</v>
+        <v>0.001016148338340419</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>0.002362593776477647</v>
+        <v>0.002351838900137252</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         <v>9</v>
       </c>
       <c r="C36" t="n">
-        <v>0.005191726513175247</v>
+        <v>0.005158111950343115</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v>10</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0107232113443282</v>
+        <v>0.01064627609145105</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         <v>11</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02064252743373656</v>
+        <v>0.0205002131684362</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>12</v>
       </c>
       <c r="C39" t="n">
-        <v>0.03712123529810048</v>
+        <v>0.03689038695410365</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
         <v>13</v>
       </c>
       <c r="C40" t="n">
-        <v>0.06226341722432225</v>
+        <v>0.06192798817807987</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         <v>14</v>
       </c>
       <c r="C41" t="n">
-        <v>0.09582669889821764</v>
+        <v>0.0954229340294396</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
         <v>15</v>
       </c>
       <c r="C42" t="n">
-        <v>0.1315540976982745</v>
+        <v>0.131215228759701</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
         <v>16</v>
       </c>
       <c r="C43" t="n">
-        <v>0.1564336735235964</v>
+        <v>0.1563246699087814</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         <v>17</v>
       </c>
       <c r="C44" t="n">
-        <v>0.1576613220800806</v>
+        <v>0.1578334297487936</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         <v>18</v>
       </c>
       <c r="C45" t="n">
-        <v>0.1330756783712803</v>
+        <v>0.1334297536534739</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         <v>19</v>
       </c>
       <c r="C46" t="n">
-        <v>0.09348888507774585</v>
+        <v>0.09388611320676336</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         <v>20</v>
       </c>
       <c r="C47" t="n">
-        <v>0.05422794849813479</v>
+        <v>0.05457043521100544</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C48" t="n">
-        <v>0.02550229070428087</v>
+        <v>0.02573685604087457</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         <v>22</v>
       </c>
       <c r="C49" t="n">
-        <v>0.009375817811305096</v>
+        <v>0.009497912622539139</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         <v>23</v>
       </c>
       <c r="C50" t="n">
-        <v>0.002516056530992395</v>
+        <v>0.002564401856591012</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>24</v>
       </c>
       <c r="C51" t="n">
-        <v>0.0004388668742248875</v>
+        <v>0.0004527712336162963</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1353,7 +1353,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1371,7 +1371,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1389,7 +1389,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1407,7 +1407,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1425,7 +1425,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1443,7 +1443,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1461,7 +1461,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1479,7 +1479,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1497,7 +1497,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1515,7 +1515,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1533,7 +1533,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1551,7 +1551,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1569,7 +1569,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1587,7 +1587,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1605,7 +1605,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1623,7 +1623,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1641,7 +1641,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1659,7 +1659,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1677,7 +1677,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1695,7 +1695,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1713,7 +1713,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1731,7 +1731,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1749,7 +1749,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1767,7 +1767,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1785,7 +1785,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1803,7 +1803,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1821,7 +1821,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1839,7 +1839,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1857,7 +1857,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1875,7 +1875,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1893,7 +1893,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1911,7 +1911,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1929,7 +1929,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1947,7 +1947,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1965,7 +1965,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1983,7 +1983,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2001,7 +2001,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2019,7 +2019,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2037,7 +2037,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2055,7 +2055,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2073,7 +2073,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2091,7 +2091,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2109,7 +2109,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2127,7 +2127,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2145,7 +2145,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2163,7 +2163,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2181,7 +2181,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2199,7 +2199,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2217,7 +2217,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2235,7 +2235,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2253,7 +2253,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2271,7 +2271,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2289,7 +2289,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2307,7 +2307,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2325,7 +2325,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2343,7 +2343,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2361,7 +2361,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2379,7 +2379,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2397,7 +2397,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2415,7 +2415,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2433,7 +2433,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2451,7 +2451,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2469,7 +2469,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2487,7 +2487,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2505,7 +2505,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2523,7 +2523,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2541,7 +2541,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2559,7 +2559,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2577,7 +2577,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2595,7 +2595,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2613,7 +2613,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2631,7 +2631,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2649,7 +2649,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2667,7 +2667,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2685,7 +2685,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Same epitope, different strain</t>
+          <t>Same peptide, different strain</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2703,7 +2703,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2721,7 +2721,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2739,7 +2739,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2757,7 +2757,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2775,7 +2775,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2793,7 +2793,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2811,7 +2811,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2829,7 +2829,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2847,7 +2847,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2865,7 +2865,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2883,7 +2883,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2901,7 +2901,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2919,7 +2919,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2937,7 +2937,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2955,7 +2955,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -2973,7 +2973,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -2991,7 +2991,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -3009,7 +3009,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -3027,7 +3027,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -3045,7 +3045,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -3063,7 +3063,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -3081,7 +3081,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -3099,7 +3099,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -3117,7 +3117,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -3135,7 +3135,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -3153,7 +3153,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -3171,7 +3171,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -3189,7 +3189,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -3207,7 +3207,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -3225,7 +3225,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -3243,7 +3243,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -3261,7 +3261,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -3279,7 +3279,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -3297,7 +3297,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -3315,7 +3315,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -3333,7 +3333,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -3351,7 +3351,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -3369,7 +3369,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -3387,7 +3387,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -3405,7 +3405,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -3423,7 +3423,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -3441,7 +3441,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -3459,7 +3459,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -3477,7 +3477,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -3495,7 +3495,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -3513,7 +3513,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -3531,7 +3531,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -3549,7 +3549,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -3567,7 +3567,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -3585,7 +3585,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Same strain, different epitope</t>
+          <t>Same strain, different peptide</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -3603,7 +3603,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -3621,7 +3621,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -3639,7 +3639,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -3657,7 +3657,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -3675,7 +3675,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -3693,7 +3693,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -3711,7 +3711,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -3729,7 +3729,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -3747,7 +3747,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -3765,7 +3765,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -3783,7 +3783,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -3801,7 +3801,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -3819,7 +3819,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -3837,7 +3837,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -3855,7 +3855,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -3873,7 +3873,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -3891,7 +3891,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -3909,7 +3909,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -3927,7 +3927,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -3945,7 +3945,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -3963,7 +3963,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -3981,7 +3981,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -3999,7 +3999,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -4017,7 +4017,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -4035,7 +4035,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -4053,7 +4053,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -4071,7 +4071,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -4089,7 +4089,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -4107,7 +4107,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -4125,7 +4125,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -4143,7 +4143,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -4161,7 +4161,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -4179,7 +4179,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -4197,7 +4197,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -4215,7 +4215,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -4233,7 +4233,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -4251,7 +4251,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -4269,7 +4269,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -4287,7 +4287,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -4305,7 +4305,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -4323,7 +4323,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -4341,7 +4341,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -4359,7 +4359,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -4377,7 +4377,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -4395,7 +4395,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -4413,7 +4413,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -4431,7 +4431,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -4449,7 +4449,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -4467,7 +4467,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -4485,7 +4485,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -4503,7 +4503,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -4521,7 +4521,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -4539,7 +4539,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -4557,7 +4557,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -4575,7 +4575,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -4593,7 +4593,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -4611,7 +4611,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -4629,7 +4629,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -4647,7 +4647,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -4665,7 +4665,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -4683,7 +4683,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -4701,7 +4701,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -4719,7 +4719,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -4737,7 +4737,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -4755,7 +4755,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -4773,7 +4773,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -4791,7 +4791,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -4809,7 +4809,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -4827,7 +4827,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -4845,7 +4845,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -4863,7 +4863,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -4881,7 +4881,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -4899,7 +4899,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -4917,7 +4917,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -4935,7 +4935,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -4953,7 +4953,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -4971,7 +4971,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -4989,7 +4989,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -5007,7 +5007,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -5025,7 +5025,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -5043,7 +5043,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -5061,7 +5061,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -5079,7 +5079,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -5097,7 +5097,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -5115,7 +5115,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -5133,7 +5133,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -5151,7 +5151,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -5169,7 +5169,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -5187,7 +5187,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -5205,7 +5205,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -5223,7 +5223,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -5241,7 +5241,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -5259,7 +5259,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -5277,7 +5277,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -5295,7 +5295,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -5313,7 +5313,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -5331,7 +5331,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -5349,7 +5349,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -5367,7 +5367,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -5385,7 +5385,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -5403,7 +5403,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -5421,7 +5421,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -5439,7 +5439,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -5457,7 +5457,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -5475,7 +5475,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -5493,7 +5493,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -5511,7 +5511,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -5529,7 +5529,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -5547,7 +5547,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -5565,7 +5565,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -5583,7 +5583,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -5601,7 +5601,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -5619,7 +5619,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -5637,7 +5637,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -5655,7 +5655,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -5673,7 +5673,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -5691,7 +5691,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -5709,7 +5709,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -5727,7 +5727,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -5745,7 +5745,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -5763,7 +5763,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -5781,7 +5781,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -5799,7 +5799,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -5817,7 +5817,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -5835,7 +5835,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -5853,7 +5853,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -5871,7 +5871,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -5889,7 +5889,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -5907,7 +5907,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -5925,7 +5925,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -5943,7 +5943,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -5961,7 +5961,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -5979,7 +5979,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -5997,7 +5997,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -6015,7 +6015,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -6033,7 +6033,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -6051,7 +6051,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -6069,7 +6069,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -6087,7 +6087,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B315" t="n">
@@ -6105,7 +6105,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B316" t="n">
@@ -6123,7 +6123,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B317" t="n">
@@ -6141,7 +6141,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B318" t="n">
@@ -6159,7 +6159,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B319" t="n">
@@ -6177,7 +6177,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B320" t="n">
@@ -6195,7 +6195,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B321" t="n">
@@ -6213,7 +6213,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B322" t="n">
@@ -6231,7 +6231,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -6249,7 +6249,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B324" t="n">
@@ -6267,7 +6267,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B325" t="n">
@@ -6285,7 +6285,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Same strain, same epitope</t>
+          <t>Same strain, same peptide</t>
         </is>
       </c>
       <c r="B326" t="n">

</xml_diff>

<commit_message>
changed names, fixed grouping logic created figures for the diss specifically
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
@@ -910,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1.730262261681266e-09</v>
+        <v>1.817426551454418e-09</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>5.109053708058755e-08</v>
+        <v>5.263527505129866e-08</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>7.151498059568239e-07</v>
+        <v>7.268241043417333e-07</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>6.026289630808105e-06</v>
+        <v>6.070467278234706e-06</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>3.361721063979729e-05</v>
+        <v>3.367318024377881e-05</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0001328756464798305</v>
+        <v>0.0001326720491835746</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         <v>6</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0004012430301734141</v>
+        <v>0.0004000812827755965</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
         <v>7</v>
       </c>
       <c r="C34" t="n">
-        <v>0.001016148338340419</v>
+        <v>0.001012869088658469</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>0.002351838900137252</v>
+        <v>0.002344433714557859</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         <v>9</v>
       </c>
       <c r="C36" t="n">
-        <v>0.005158111950343115</v>
+        <v>0.005142860321620531</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v>10</v>
       </c>
       <c r="C37" t="n">
-        <v>0.01064627609145105</v>
+        <v>0.01061639260130365</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         <v>11</v>
       </c>
       <c r="C38" t="n">
-        <v>0.0205002131684362</v>
+        <v>0.02044611959513187</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>12</v>
       </c>
       <c r="C39" t="n">
-        <v>0.03689038695410365</v>
+        <v>0.036806208070158</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
         <v>13</v>
       </c>
       <c r="C40" t="n">
-        <v>0.06192798817807987</v>
+        <v>0.06181695769759248</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         <v>14</v>
       </c>
       <c r="C41" t="n">
-        <v>0.0954229340294396</v>
+        <v>0.09529438342105105</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
         <v>15</v>
       </c>
       <c r="C42" t="n">
-        <v>0.131215228759701</v>
+        <v>0.1310887197683009</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
         <v>16</v>
       </c>
       <c r="C43" t="n">
-        <v>0.1563246699087814</v>
+        <v>0.1562414269860764</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         <v>17</v>
       </c>
       <c r="C44" t="n">
-        <v>0.1578334297487936</v>
+        <v>0.1578434105559419</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         <v>18</v>
       </c>
       <c r="C45" t="n">
-        <v>0.1334297536534739</v>
+        <v>0.1335513887633853</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         <v>19</v>
       </c>
       <c r="C46" t="n">
-        <v>0.09388611320676336</v>
+        <v>0.094072177567136</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         <v>20</v>
       </c>
       <c r="C47" t="n">
-        <v>0.05457043521100544</v>
+        <v>0.05473956519993334</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C48" t="n">
-        <v>0.02573685604087457</v>
+        <v>0.0258396950390542</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         <v>22</v>
       </c>
       <c r="C49" t="n">
-        <v>0.009497912622539139</v>
+        <v>0.009541469192245683</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         <v>23</v>
       </c>
       <c r="C50" t="n">
-        <v>0.002564401856591012</v>
+        <v>0.002575410673112297</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>24</v>
       </c>
       <c r="C51" t="n">
-        <v>0.0004527712336162963</v>
+        <v>0.0004532334884528062</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
made more histograms and then also made my code actually readable (thats a bit of an exagerration) made the documentation somewhat coherent sui
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
@@ -910,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1.817426551454418e-09</v>
+        <v>1.757126109274727e-09</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>5.263527505129866e-08</v>
+        <v>5.131808961523976e-08</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>7.268241043417333e-07</v>
+        <v>7.156233511370521e-07</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>6.070467278234706e-06</v>
+        <v>6.023531616724019e-06</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>3.367318024377881e-05</v>
+        <v>3.359717513603453e-05</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0001326720491835746</v>
+        <v>0.0001327962944614731</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         <v>6</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0004000812827755965</v>
+        <v>0.0004008947119308098</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
         <v>7</v>
       </c>
       <c r="C34" t="n">
-        <v>0.001012869088658469</v>
+        <v>0.001014929378788123</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>0.002344433714557859</v>
+        <v>0.002349115078962906</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         <v>9</v>
       </c>
       <c r="C36" t="n">
-        <v>0.005142860321620531</v>
+        <v>0.005154352325628063</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v>10</v>
       </c>
       <c r="C37" t="n">
-        <v>0.01061639260130365</v>
+        <v>0.01064324858491328</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         <v>11</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02044611959513187</v>
+        <v>0.02049950936854881</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>12</v>
       </c>
       <c r="C39" t="n">
-        <v>0.036806208070158</v>
+        <v>0.03689345465017832</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
         <v>13</v>
       </c>
       <c r="C40" t="n">
-        <v>0.06181695769759248</v>
+        <v>0.06193702609246685</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         <v>14</v>
       </c>
       <c r="C41" t="n">
-        <v>0.09529438342105105</v>
+        <v>0.09543821747932225</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
         <v>15</v>
       </c>
       <c r="C42" t="n">
-        <v>0.1310887197683009</v>
+        <v>0.131232937801542</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
         <v>16</v>
       </c>
       <c r="C43" t="n">
-        <v>0.1562414269860764</v>
+        <v>0.1563409423665826</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         <v>17</v>
       </c>
       <c r="C44" t="n">
-        <v>0.1578434105559419</v>
+        <v>0.157846659194112</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         <v>18</v>
       </c>
       <c r="C45" t="n">
-        <v>0.1335513887633853</v>
+        <v>0.1334380293602676</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         <v>19</v>
       </c>
       <c r="C46" t="n">
-        <v>0.094072177567136</v>
+        <v>0.09388425718411003</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         <v>20</v>
       </c>
       <c r="C47" t="n">
-        <v>0.05473956519993334</v>
+        <v>0.05455526882616727</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C48" t="n">
-        <v>0.0258396950390542</v>
+        <v>0.02571436349585139</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         <v>22</v>
       </c>
       <c r="C49" t="n">
-        <v>0.009541469192245683</v>
+        <v>0.009479689992221414</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         <v>23</v>
       </c>
       <c r="C50" t="n">
-        <v>0.002575410673112297</v>
+        <v>0.002555067346220661</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>24</v>
       </c>
       <c r="C51" t="n">
-        <v>0.0004532334884528062</v>
+        <v>0.0004488510624045481</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
oops accidentally got rid of pre immune on the v gene dependency graphs and then also added dextramer vs dextramer plots and also did the within dextramer normality tests and then also did the tcrbeta normalities and then also did the within clonotype per cell counts with proportions per cell sui and then just reran everything sui
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
@@ -910,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1.757126109274727e-09</v>
+        <v>1.764780103097454e-09</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>5.131808961523976e-08</v>
+        <v>5.119472109405238e-08</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>7.156233511370521e-07</v>
+        <v>7.11045747463041e-07</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>6.023531616724019e-06</v>
+        <v>5.974058472613702e-06</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>3.359717513603453e-05</v>
+        <v>3.330189641680093e-05</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0001327962944614731</v>
+        <v>0.0001317051289035694</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         <v>6</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0004008947119308098</v>
+        <v>0.0003982588148489614</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
         <v>7</v>
       </c>
       <c r="C34" t="n">
-        <v>0.001014929378788123</v>
+        <v>0.001010174067788207</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>0.002349115078962906</v>
+        <v>0.002341202315420117</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         <v>9</v>
       </c>
       <c r="C36" t="n">
-        <v>0.005154352325628063</v>
+        <v>0.005141361926188636</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v>10</v>
       </c>
       <c r="C37" t="n">
-        <v>0.01064324858491328</v>
+        <v>0.01062563376925515</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         <v>11</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02049950936854881</v>
+        <v>0.02048525553849773</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>12</v>
       </c>
       <c r="C39" t="n">
-        <v>0.03689345465017832</v>
+        <v>0.03689828187414144</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
         <v>13</v>
       </c>
       <c r="C40" t="n">
-        <v>0.06193702609246685</v>
+        <v>0.06197281856836279</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         <v>14</v>
       </c>
       <c r="C41" t="n">
-        <v>0.09543821747932225</v>
+        <v>0.09548982229443166</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
         <v>15</v>
       </c>
       <c r="C42" t="n">
-        <v>0.131232937801542</v>
+        <v>0.1312511493923275</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
         <v>16</v>
       </c>
       <c r="C43" t="n">
-        <v>0.1563409423665826</v>
+        <v>0.1562830612315206</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         <v>17</v>
       </c>
       <c r="C44" t="n">
-        <v>0.157846659194112</v>
+        <v>0.1577362266340091</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         <v>18</v>
       </c>
       <c r="C45" t="n">
-        <v>0.1334380293602676</v>
+        <v>0.1333580648721567</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         <v>19</v>
       </c>
       <c r="C46" t="n">
-        <v>0.09388425718411003</v>
+        <v>0.09388791417267053</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         <v>20</v>
       </c>
       <c r="C47" t="n">
-        <v>0.05455526882616727</v>
+        <v>0.0546160786196116</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C48" t="n">
-        <v>0.02571436349585139</v>
+        <v>0.0257816118038653</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         <v>22</v>
       </c>
       <c r="C49" t="n">
-        <v>0.009479689992221414</v>
+        <v>0.009523828040939299</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         <v>23</v>
       </c>
       <c r="C50" t="n">
-        <v>0.002555067346220661</v>
+        <v>0.002573440929795747</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>24</v>
       </c>
       <c r="C51" t="n">
-        <v>0.0004488510624045481</v>
+        <v>0.0004540700451272729</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Reran comparison 1 stuff with the seaborn context style 'talk'
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
@@ -910,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1.764780103097454e-09</v>
+        <v>1.785249376105226e-09</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>5.119472109405238e-08</v>
+        <v>5.185314946034674e-08</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>7.11045747463041e-07</v>
+        <v>7.20174082828375e-07</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>5.974058472613702e-06</v>
+        <v>6.050856019144276e-06</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>3.330189641680093e-05</v>
+        <v>3.372543704873797e-05</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0001317051289035694</v>
+        <v>0.0001332687124505398</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         <v>6</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0003982588148489614</v>
+        <v>0.0004024256245162271</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
         <v>7</v>
       </c>
       <c r="C34" t="n">
-        <v>0.001010174067788207</v>
+        <v>0.00101968234792391</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>0.002341202315420117</v>
+        <v>0.002362470323225413</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         <v>9</v>
       </c>
       <c r="C36" t="n">
-        <v>0.005141361926188636</v>
+        <v>0.005186406265150699</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v>10</v>
       </c>
       <c r="C37" t="n">
-        <v>0.01062563376925515</v>
+        <v>0.0107113856874115</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         <v>11</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02048525553849773</v>
+        <v>0.02063382982938205</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>12</v>
       </c>
       <c r="C39" t="n">
-        <v>0.03689828187414144</v>
+        <v>0.0371343380435009</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
         <v>13</v>
       </c>
       <c r="C40" t="n">
-        <v>0.06197281856836279</v>
+        <v>0.06230640887290947</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         <v>14</v>
       </c>
       <c r="C41" t="n">
-        <v>0.09548982229443166</v>
+        <v>0.09588800494358353</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
         <v>15</v>
       </c>
       <c r="C42" t="n">
-        <v>0.1312511493923275</v>
+        <v>0.1316155028862812</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
         <v>16</v>
       </c>
       <c r="C43" t="n">
-        <v>0.1562830612315206</v>
+        <v>0.1564688608179386</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         <v>17</v>
       </c>
       <c r="C44" t="n">
-        <v>0.1577362266340091</v>
+        <v>0.1576364750419315</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         <v>18</v>
       </c>
       <c r="C45" t="n">
-        <v>0.1333580648721567</v>
+        <v>0.1329977616414301</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         <v>19</v>
       </c>
       <c r="C46" t="n">
-        <v>0.09388791417267053</v>
+        <v>0.09341468583359039</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         <v>20</v>
       </c>
       <c r="C47" t="n">
-        <v>0.0546160786196116</v>
+        <v>0.054195200750385</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C48" t="n">
-        <v>0.0257816118038653</v>
+        <v>0.02550048936338579</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         <v>22</v>
       </c>
       <c r="C49" t="n">
-        <v>0.009523828040939299</v>
+        <v>0.009385692000130813</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         <v>23</v>
       </c>
       <c r="C50" t="n">
-        <v>0.002573440929795747</v>
+        <v>0.002524213943101336</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>24</v>
       </c>
       <c r="C51" t="n">
-        <v>0.0004540700451272729</v>
+        <v>0.0004423469662214248</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Yeah i made a typo which meant the same strain same peptide columns in the hierarchy decomp became grey
</commit_message>
<xml_diff>
--- a/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
+++ b/Final_Figures_and_Sheets_Singleset/H-2Kb_pcDelta_paired_convolved.xlsx
@@ -910,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>1.785249376105226e-09</v>
+        <v>1.791053583918167e-09</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>5.185314946034674e-08</v>
+        <v>5.221275590998393e-08</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>7.20174082828375e-07</v>
+        <v>7.252099567970312e-07</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>6.050856019144276e-06</v>
+        <v>6.079544426065497e-06</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>3.372543704873797e-05</v>
+        <v>3.377295404876139e-05</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0001332687124505398</v>
+        <v>0.0001330539592174154</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
         <v>6</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0004024256245162271</v>
+        <v>0.000401057508413464</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
         <v>7</v>
       </c>
       <c r="C34" t="n">
-        <v>0.00101968234792391</v>
+        <v>0.001015589385331026</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1054,7 +1054,7 @@
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>0.002362470323225413</v>
+        <v>0.002352922918548637</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         <v>9</v>
       </c>
       <c r="C36" t="n">
-        <v>0.005186406265150699</v>
+        <v>0.005166327616293889</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         <v>10</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0107113856874115</v>
+        <v>0.01067001845226793</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         <v>11</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02063382982938205</v>
+        <v>0.02054492792922992</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>12</v>
       </c>
       <c r="C39" t="n">
-        <v>0.0371343380435009</v>
+        <v>0.03694944713292649</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
         <v>13</v>
       </c>
       <c r="C40" t="n">
-        <v>0.06230640887290947</v>
+        <v>0.0619762450414874</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         <v>14</v>
       </c>
       <c r="C41" t="n">
-        <v>0.09588800494358353</v>
+        <v>0.09541362438584233</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
         <v>15</v>
       </c>
       <c r="C42" t="n">
-        <v>0.1316155028862812</v>
+        <v>0.1310997545888273</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
         <v>16</v>
       </c>
       <c r="C43" t="n">
-        <v>0.1564688608179386</v>
+        <v>0.1561095292882388</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         <v>17</v>
       </c>
       <c r="C44" t="n">
-        <v>0.1576364750419315</v>
+        <v>0.1576142790697581</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         <v>18</v>
       </c>
       <c r="C45" t="n">
-        <v>0.1329977616414301</v>
+        <v>0.1333303912640797</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         <v>19</v>
       </c>
       <c r="C46" t="n">
-        <v>0.09341468583359039</v>
+        <v>0.09394933136542018</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
         <v>20</v>
       </c>
       <c r="C47" t="n">
-        <v>0.054195200750385</v>
+        <v>0.05472393789924955</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C48" t="n">
-        <v>0.02550048936338579</v>
+        <v>0.02587580279935197</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         <v>22</v>
       </c>
       <c r="C49" t="n">
-        <v>0.009385692000130813</v>
+        <v>0.009578501111134943</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1324,7 +1324,7 @@
         <v>23</v>
       </c>
       <c r="C50" t="n">
-        <v>0.002524213943101336</v>
+        <v>0.002595490704223167</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1342,7 +1342,7 @@
         <v>24</v>
       </c>
       <c r="C51" t="n">
-        <v>0.0004423469662214248</v>
+        <v>0.0004591358679167952</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>

</xml_diff>